<commit_message>
updated experiment excel template
</commit_message>
<xml_diff>
--- a/assets/empty/faang_experiment.xlsx
+++ b/assets/empty/faang_experiment.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yroochun/Projects/FAANG_TEMPLATES/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61370CF9-10A7-B644-A8B6-A3FD9ED7A238}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{162005C1-2060-EC43-859C-259687B4C528}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28800" yWindow="600" windowWidth="38400" windowHeight="19060" activeTab="15" xr2:uid="{58DBCFEB-F75F-A348-9496-13E962F9C8F7}"/>
+    <workbookView xWindow="28800" yWindow="0" windowWidth="38400" windowHeight="21600" activeTab="16" xr2:uid="{58DBCFEB-F75F-A348-9496-13E962F9C8F7}"/>
   </bookViews>
   <sheets>
     <sheet name="submission" sheetId="13" r:id="rId1"/>
@@ -53,7 +53,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="718" uniqueCount="349">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="701" uniqueCount="348">
   <si>
     <t>Sample Descriptor</t>
   </si>
@@ -1031,9 +1031,6 @@
   </si>
   <si>
     <t>snATAC-seq</t>
-  </si>
-  <si>
-    <t>scATAC-seq assay type</t>
   </si>
   <si>
     <t>scATAC-seq sample storage processing</t>
@@ -2468,34 +2465,34 @@
         <v>82</v>
       </c>
       <c r="AC1" s="9" t="s">
+        <v>339</v>
+      </c>
+      <c r="AD1" s="9" t="s">
         <v>340</v>
       </c>
-      <c r="AD1" s="9" t="s">
+      <c r="AE1" s="9" t="s">
         <v>341</v>
       </c>
-      <c r="AE1" s="9" t="s">
+      <c r="AF1" s="9" t="s">
         <v>342</v>
       </c>
-      <c r="AF1" s="9" t="s">
+      <c r="AG1" s="9" t="s">
         <v>343</v>
       </c>
-      <c r="AG1" s="9" t="s">
+      <c r="AH1" s="9" t="s">
         <v>344</v>
       </c>
-      <c r="AH1" s="9" t="s">
+      <c r="AI1" s="9" t="s">
         <v>345</v>
       </c>
-      <c r="AI1" s="9" t="s">
+      <c r="AJ1" s="9" t="s">
         <v>346</v>
-      </c>
-      <c r="AJ1" s="9" t="s">
-        <v>347</v>
       </c>
       <c r="AK1" s="9" t="s">
         <v>309</v>
       </c>
       <c r="AL1" s="9" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="AM1" s="9"/>
     </row>
@@ -2531,7 +2528,7 @@
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="4">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{9DAD5BB5-2950-0048-BD7E-9416EB636803}">
           <x14:formula1>
-            <xm:f>faang_field_values!$C$22:$R$22</xm:f>
+            <xm:f>faang_field_values!$C$1:$R$1</xm:f>
           </x14:formula1>
           <xm:sqref>E2</xm:sqref>
         </x14:dataValidation>
@@ -3816,61 +3813,11 @@
     </row>
     <row r="21" spans="1:55" ht="15.75" customHeight="1"/>
     <row r="22" spans="1:55" ht="15.75" customHeight="1">
-      <c r="A22" s="5" t="s">
-        <v>326</v>
-      </c>
-      <c r="C22" t="s">
-        <v>22</v>
-      </c>
-      <c r="D22" t="s">
-        <v>23</v>
-      </c>
-      <c r="E22" t="s">
-        <v>32</v>
-      </c>
-      <c r="F22" t="s">
-        <v>31</v>
-      </c>
-      <c r="G22" t="s">
-        <v>24</v>
-      </c>
-      <c r="H22" t="s">
-        <v>25</v>
-      </c>
-      <c r="I22" t="s">
-        <v>26</v>
-      </c>
-      <c r="J22" t="s">
-        <v>27</v>
-      </c>
-      <c r="K22" t="s">
-        <v>28</v>
-      </c>
-      <c r="L22" t="s">
-        <v>29</v>
-      </c>
-      <c r="M22" t="s">
-        <v>30</v>
-      </c>
-      <c r="N22" t="s">
-        <v>15</v>
-      </c>
-      <c r="O22" t="s">
-        <v>324</v>
-      </c>
-      <c r="P22" t="s">
-        <v>303</v>
-      </c>
-      <c r="Q22" t="s">
-        <v>325</v>
-      </c>
-      <c r="R22" t="s">
-        <v>76</v>
-      </c>
+      <c r="A22" s="5"/>
     </row>
     <row r="23" spans="1:55" ht="15.75" customHeight="1">
       <c r="A23" s="5" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C23" t="s">
         <v>20</v>
@@ -3902,42 +3849,42 @@
     </row>
     <row r="24" spans="1:55" ht="15.75" customHeight="1">
       <c r="A24" s="5" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="C24" t="s">
+        <v>327</v>
+      </c>
+      <c r="D24" t="s">
         <v>328</v>
       </c>
-      <c r="D24" t="s">
+      <c r="E24" t="s">
         <v>329</v>
       </c>
-      <c r="E24" t="s">
+      <c r="F24" t="s">
         <v>330</v>
       </c>
-      <c r="F24" t="s">
+      <c r="G24" t="s">
         <v>331</v>
       </c>
-      <c r="G24" t="s">
+      <c r="H24" t="s">
         <v>332</v>
       </c>
-      <c r="H24" t="s">
+      <c r="I24" t="s">
         <v>333</v>
       </c>
-      <c r="I24" t="s">
+      <c r="J24" t="s">
         <v>334</v>
       </c>
-      <c r="J24" t="s">
+      <c r="K24" t="s">
         <v>335</v>
       </c>
-      <c r="K24" t="s">
+      <c r="L24" t="s">
         <v>336</v>
-      </c>
-      <c r="L24" t="s">
-        <v>337</v>
       </c>
     </row>
     <row r="25" spans="1:55" ht="15.75" customHeight="1">
       <c r="A25" s="5" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="C25" t="s">
         <v>34</v>

</xml_diff>